<commit_message>
Support premium double-mode upload and download for cloud environments
</commit_message>
<xml_diff>
--- a/TEST.xlsx
+++ b/TEST.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
   <si>
     <t>상품명</t>
   </si>
@@ -30,130 +30,220 @@
     <t>정제된 상품명</t>
   </si>
   <si>
-    <t>큐티 고양이발 자</t>
-  </si>
-  <si>
-    <t>길이조절형 북엔드</t>
-  </si>
-  <si>
-    <t>만능 물때지우개</t>
-  </si>
-  <si>
-    <t>다용도 미니 공예용 망치 손잡이 1p</t>
-  </si>
-  <si>
-    <t>동물 점착 메모지 20매</t>
-  </si>
-  <si>
-    <t>부착형 우산꽂이</t>
-  </si>
-  <si>
-    <t>가죽 키링</t>
-  </si>
-  <si>
-    <t>멍멍이 휴대용 접이식 장바구니 1p</t>
-  </si>
-  <si>
-    <t>토끼귀 리모컨 커버</t>
-  </si>
-  <si>
-    <t>A4 우드 클립보드</t>
-  </si>
-  <si>
-    <t>색소폰 하네스 스트랩</t>
-  </si>
-  <si>
-    <t>접이식 양면 스텐 미니 손거울 열쇠고리</t>
-  </si>
-  <si>
-    <t>컬러 별모양 스티커 10p</t>
-  </si>
-  <si>
-    <t>동물 세안 헤어밴드</t>
-  </si>
-  <si>
-    <t>고양이 발바닥 모양 반려동물 캔따개</t>
-  </si>
-  <si>
-    <t>쇼클립(집게대/봉50/클립)(3958)</t>
-  </si>
-  <si>
-    <t>쇼케이스B7(양면/세로)(0686)</t>
-  </si>
-  <si>
-    <t>단면POP꽂이 L-1515</t>
-  </si>
-  <si>
-    <t>주유혼유방지 링커버</t>
-  </si>
-  <si>
-    <t>피오르니 아로마 케어 디퓨저 200ml</t>
-  </si>
-  <si>
-    <t>피오르니 우드볼 디퓨저 200ml</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500382</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500383</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500384</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500386</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500387</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500388</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500389</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500391</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500392</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500396</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500397</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500398</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500399</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500400</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500402</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500404</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500406</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500410</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500413</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500415</t>
-  </si>
-  <si>
-    <t>https://www.new79dome.com/shop/item.php?it_id=500416</t>
+    <t>밀워키 워터펌프플라이어첼라 48 22 62 12</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57821&amp;code=</t>
+  </si>
+  <si>
+    <t>밀워키 워터펌프플라이어첼라 48 22 62 10</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57820&amp;code=</t>
+  </si>
+  <si>
+    <t>밀워키 플라이어첼라 48 22 63 12</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57818&amp;code=</t>
+  </si>
+  <si>
+    <t>밀워키 플라이어첼라 48 22 63 10</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57817&amp;code=</t>
+  </si>
+  <si>
+    <t>밀워키 양날토션비트 48 32 4361 65mm 10pcs PH2</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57811&amp;code=</t>
+  </si>
+  <si>
+    <t>9080 부직포 양면테이프 50mm x 50M</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57798&amp;code=</t>
+  </si>
+  <si>
+    <t>9080 부직포 양면테이프 20mm x 50M</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57796&amp;code=</t>
+  </si>
+  <si>
+    <t>961 수세미 패드 홀더 수세미손잡이</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57793&amp;code=</t>
+  </si>
+  <si>
+    <t>귀마개 케이스 귀마개보관함</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57788&amp;code=</t>
+  </si>
+  <si>
+    <t>경량형 귀덮개 X1A 청력 보호구</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57783&amp;code=</t>
+  </si>
+  <si>
+    <t>철제 실리콘 건 철재질</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57773&amp;code=</t>
+  </si>
+  <si>
+    <t>실리콘 헤라 마감용헤라 대 43mm</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57772&amp;code=</t>
+  </si>
+  <si>
+    <t>실리콘 헤라 마감용헤라 중 36mm</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57771&amp;code=</t>
+  </si>
+  <si>
+    <t>실리콘 헤라 마감용헤라 소 28mm</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57770&amp;code=</t>
+  </si>
+  <si>
+    <t>실리콘 헤라 마감용헤라 미니 20mm</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57769&amp;code=</t>
+  </si>
+  <si>
+    <t>에어타카 KTF 50NA KTF 50N후속 F핀사용</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57768&amp;code=</t>
+  </si>
+  <si>
+    <t>직소 GST8000E 710W 목재용날포함 오비탈기능</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57767&amp;code=</t>
+  </si>
+  <si>
+    <t>밀워키 충전직소 M18 BJS 0C0 18V 본체 베어툴</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57761&amp;code=</t>
+  </si>
+  <si>
+    <t>트리머날6mm 440</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57754&amp;code=</t>
+  </si>
+  <si>
+    <t>스탠리 사각샌더 SS24 240W 먼지주머니포함</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57752&amp;code=</t>
+  </si>
+  <si>
+    <t>먼지주머니122852 0 LS1040S용</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57751&amp;code=</t>
+  </si>
+  <si>
+    <t>원형톱 CS235 20 9 톱날포함 CS 9A후속</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57749&amp;code=</t>
+  </si>
+  <si>
+    <t>가이드레일FSN800</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57748&amp;code=</t>
+  </si>
+  <si>
+    <t>원형톱가이드MRG L1000</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57732&amp;code=</t>
+  </si>
+  <si>
+    <t>대영톱 전정톱350mm</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57725&amp;code=</t>
+  </si>
+  <si>
+    <t>대영톱 전정톱300mm</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57724&amp;code=</t>
+  </si>
+  <si>
+    <t>대영톱 전정톱240mm</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57722&amp;code=</t>
+  </si>
+  <si>
+    <t>ARS 접톱PM 21</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57720&amp;code=</t>
+  </si>
+  <si>
+    <t>MKK 목공용톱HMK 190</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57719&amp;code=</t>
+  </si>
+  <si>
+    <t>대영톱 전정톱500</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57707&amp;code=</t>
+  </si>
+  <si>
+    <t>백마 목공톱 등대기톱 TH 104 270mm</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57703&amp;code=</t>
+  </si>
+  <si>
+    <t>백마 전지톱G 30 300mm</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57702&amp;code=</t>
+  </si>
+  <si>
+    <t>백마 산림톱TH 2000 360mm</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57700&amp;code=</t>
+  </si>
+  <si>
+    <t>OKITO 핸드샌더GM HS20 20PCS</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57694&amp;code=</t>
+  </si>
+  <si>
+    <t>직소날세트B 06482 B 52 5PCS</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57691&amp;code=</t>
+  </si>
+  <si>
+    <t>베세이 L 클램프 목공용 KRE80 2K</t>
+  </si>
+  <si>
+    <t>https://www.3mro.co.kr/shop/item.php?it_id=57688&amp;code=</t>
   </si>
 </sst>
 </file>
@@ -501,7 +591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AS22"/>
+  <dimension ref="A1:AS37"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -525,189 +615,309 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="AS2" s="1"/>
     </row>
     <row r="3" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="AS3" s="1"/>
     </row>
     <row r="4" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="AS4" s="1"/>
     </row>
     <row r="5" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="AS5" s="1"/>
     </row>
     <row r="6" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="AS6" s="1"/>
     </row>
     <row r="7" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="AS7" s="1"/>
     </row>
     <row r="8" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="AS8" s="1"/>
     </row>
     <row r="9" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="AS9" s="1"/>
     </row>
     <row r="10" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="AS10" s="1"/>
     </row>
     <row r="11" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="AS11" s="1"/>
     </row>
     <row r="12" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="B12" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="AS12" s="1"/>
     </row>
     <row r="13" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="AS13" s="1"/>
     </row>
     <row r="14" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="AS14" s="1"/>
     </row>
     <row r="15" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="B15" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="AS15" s="1"/>
     </row>
     <row r="16" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="B16" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="AS16" s="1"/>
     </row>
     <row r="17" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="B17" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="AS17" s="1"/>
     </row>
     <row r="18" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="AS18" s="1"/>
     </row>
     <row r="19" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="B19" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="AS19" s="1"/>
     </row>
     <row r="20" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="AS20" s="1"/>
     </row>
     <row r="21" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="B21" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="AS21" s="1"/>
     </row>
     <row r="22" spans="1:45" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="B22" t="s">
         <v>44</v>
       </c>
       <c r="AS22" s="1"/>
+    </row>
+    <row r="23" spans="1:45" x14ac:dyDescent="0.4">
+      <c r="A23" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" spans="1:45" x14ac:dyDescent="0.4">
+      <c r="A24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="25" spans="1:45" x14ac:dyDescent="0.4">
+      <c r="A25" t="s">
+        <v>49</v>
+      </c>
+      <c r="B25" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="1:45" x14ac:dyDescent="0.4">
+      <c r="A26" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:45" x14ac:dyDescent="0.4">
+      <c r="A27" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="28" spans="1:45" x14ac:dyDescent="0.4">
+      <c r="A28" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="29" spans="1:45" x14ac:dyDescent="0.4">
+      <c r="A29" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="30" spans="1:45" x14ac:dyDescent="0.4">
+      <c r="A30" t="s">
+        <v>59</v>
+      </c>
+      <c r="B30" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31" spans="1:45" x14ac:dyDescent="0.4">
+      <c r="A31" t="s">
+        <v>61</v>
+      </c>
+      <c r="B31" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="32" spans="1:45" x14ac:dyDescent="0.4">
+      <c r="A32" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A33" t="s">
+        <v>65</v>
+      </c>
+      <c r="B33" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A34" t="s">
+        <v>67</v>
+      </c>
+      <c r="B34" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A35" t="s">
+        <v>69</v>
+      </c>
+      <c r="B35" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A36" t="s">
+        <v>71</v>
+      </c>
+      <c r="B36" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B37" t="s">
+        <v>74</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>